<commit_message>
Adicionar espectrogramas nos picos de vocalização (aba Espectrogramas).
PNG de arquivos longos passa a ser a janela de 60 s com mais eventos, não os primeiros 60 s. O Excel provisório embute o recorte de escuta 30:45 com os picos marcados — validação humana, não um PNG por evento do lote.

Co-authored-by: Antonio Junior <antoniocfjr@icloud.com>
</commit_message>
<xml_diff>
--- a/reports/relatorio_provisorio.xlsx
+++ b/reports/relatorio_provisorio.xlsx
@@ -14,7 +14,8 @@
     <sheet name="Por hora" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Por mês" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Ouvir" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Parâmetros" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Espectrogramas" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Parâmetros" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Arquivos'!$A$3:$G$78</definedName>
@@ -138,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -213,6 +214,12 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -574,6 +581,86 @@
 </wsDr>
 </file>
 
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6096000" cy="3267075"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6096000" cy="3267075"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6096000" cy="3267075"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -899,7 +986,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Este livro é PROVISÓRIO: serve para a aluna abrir, enviar por e-mail e usar no rascunho da tese. Não substitui a lista completa de eventos (output/resultado.xlsx, ~7 MB, gitignored). Não houve escuta sistemática nem PNG por arquivo (lote com --no-spectrogram).</t>
+          <t>Este livro é PROVISÓRIO: serve para a aluna abrir, enviar por e-mail e usar no rascunho da tese. Não substitui a lista completa de eventos (output/resultado.xlsx, ~7 MB, gitignored). A aba Espectrogramas traz o recorte de escuta da madrugada com os picos marcados (validação humana). Não há um PNG por evento do lote (isso seriam ~150 mil imagens).</t>
         </is>
       </c>
     </row>
@@ -959,7 +1046,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>O que a tese pode afirmar: docs/PRECISAO_E_LIMITES.md. Como ler Excel/JSON completos: docs/COMO_LER_OS_RESULTADOS.md. Parâmetros: aba Parâmetros e src/bioacoustics/config.py. Totais enxutos: reports/campo_resumo.json.</t>
+          <t>O que a tese pode afirmar: docs/PRECISAO_E_LIMITES.md. Como ler Excel/JSON completos: docs/COMO_LER_OS_RESULTADOS.md. Parâmetros: aba Parâmetros e src/bioacoustics/config.py. Totais enxutos: reports/campo_resumo.json. PNG de validação: aba Espectrogramas e reports/espectrogramas/.</t>
         </is>
       </c>
     </row>
@@ -971,7 +1058,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>python3 scripts/export_relatorio_provisorio.py  (gerado 2026-09-01 20:08 UTC). 64 eventos do recorte listados na aba Ouvir (extraídos de output/resultado.json).</t>
+          <t>python3 scripts/export_relatorio_provisorio.py  (gerado 2026-09-02 13:04 UTC). 64 eventos do recorte listados na aba Ouvir (extraídos de output/resultado.json).</t>
         </is>
       </c>
     </row>
@@ -4380,7 +4467,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Recorte de validação humana (já escolhido). PROVISÓRIO: a escuta ainda não foi feita neste lote. Confirmar espécie no ouvido antes de discutir a manhã densa.</t>
+          <t>Recorte de validação humana (já escolhido). PROVISÓRIO: a escuta ainda não foi feita neste lote. Confirmar espécie no ouvido antes de discutir a manhã densa. Espectrograma deste minuto: aba Espectrogramas.</t>
         </is>
       </c>
       <c r="B2" s="7" t="n"/>
@@ -4506,7 +4593,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Abrir o WAV no VLC/Audacity, ir a 30:45, ouvir um minuto com fones. A pergunta é: soa como o anúncio do CEAES 2, ou é outro som na banda?</t>
+          <t>Abrir o WAV no VLC/Audacity, ir a 30:45, ouvir um minuto com fones. A pergunta é: soa como o anúncio do CEAES 2, ou é outro som na banda? O espectrograma deste minuto (picos marcados) está na aba Espectrogramas.</t>
         </is>
       </c>
     </row>
@@ -6181,6 +6268,169 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="88" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PROVISÓRIO — eventos acústicos na banda calibrada 2,6–3,2 kHz; não é censo de machos nem prova de espécie em cada linha.</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Validação humana, não o método de contagem. O lote de campo não gerou um PNG por evento (seriam 149 962 imagens). Aqui só o recorte de escuta da madrugada (30:45) com os picos já encontrados marcados em verde, mais um zoom no pico mais forte. Em arquivos longos o PNG do pipeline passa a ser a janela de 60 s com mais picos, não os primeiros 60 s. Ficheiros: reports/espectrogramas/.</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n"/>
+      <c r="C2" s="7" t="n"/>
+      <c r="D2" s="7" t="n"/>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Figura</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Ficheiro</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Legenda</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>reports/espectrogramas/R20241012-041002_30m45s.png</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>embutida</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>R20241012-041002.WAV — 30:45–31:45 (04:40) — picos de vocalização. Recorte de escuta já combinado (64 eventos, ~2,93 kHz). Círculos verdes = eventos do lote, não uma recontagem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>reports/espectrogramas/R20241012-041002_pico_1854s.png</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>embutida</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Zoom ~8 s no pico mais forte deste minuto (~1853,65 s, 2928 Hz). Só para conferir a forma do canto; o método de contagem continua a ser a matriz numérica da STFT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>reports/espectrogramas/R20241012-091022_densest_60s.png</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>embutida</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>R20241012-091022.WAV — janela de 60 s mais densa — só depois da madrugada. Não começar a validação por este ficheiro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Regenerar PNGs (máquina com o WAV de campo e output/resultado.json): python3 scripts/export_espectrogramas_validacao.py  depois  python3 scripts/export_relatorio_provisorio.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>R20241012-041002.WAV — 30:45–31:45 (04:40) — picos de vocalização. Recorte de escuta já combinado (64 eventos, ~2,93 kHz). Círculos verdes = eventos do lote, não uma recontagem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="267" customHeight="1"/>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>Zoom ~8 s no pico mais forte deste minuto (~1853,65 s, 2928 Hz). Só para conferir a forma do canto; o método de contagem continua a ser a matriz numérica da STFT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="267" customHeight="1"/>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>R20241012-091022.WAV — janela de 60 s mais densa — só depois da madrugada. Não começar a validação por este ficheiro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="267" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00833C0C"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6225,7 +6475,7 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>sample_rate</t>
         </is>
@@ -6240,7 +6490,7 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t>lowcut_hz</t>
         </is>
@@ -6255,7 +6505,7 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="28" t="inlineStr">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>highcut_hz</t>
         </is>
@@ -6270,7 +6520,7 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="A7" s="30" t="inlineStr">
         <is>
           <t>filter_order</t>
         </is>
@@ -6285,7 +6535,7 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>n_fft</t>
         </is>
@@ -6300,7 +6550,7 @@
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t>hop_length</t>
         </is>
@@ -6315,7 +6565,7 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="28" t="inlineStr">
+      <c r="A10" s="30" t="inlineStr">
         <is>
           <t>use_noise_reduction</t>
         </is>
@@ -6332,7 +6582,7 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="28" t="inlineStr">
+      <c r="A11" s="30" t="inlineStr">
         <is>
           <t>noise_reduce_prop_decrease</t>
         </is>
@@ -6347,7 +6597,7 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="30" t="inlineStr">
         <is>
           <t>threshold_k</t>
         </is>
@@ -6362,7 +6612,7 @@
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="29" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>min_peak_distance_s</t>
         </is>
@@ -6370,14 +6620,14 @@
       <c r="B13" s="16" t="n">
         <v>0.15</v>
       </c>
-      <c r="C13" s="30" t="inlineStr">
+      <c r="C13" s="32" t="inlineStr">
         <is>
           <t>Declarado em DetectionConfig; NÃO é usado em detect_events.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t>event_merge_gap_s</t>
         </is>
@@ -6392,7 +6642,7 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="30" t="inlineStr">
         <is>
           <t>min_event_duration_s</t>
         </is>
@@ -6407,7 +6657,7 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="28" t="inlineStr">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>freq_separation_hz</t>
         </is>
@@ -6422,7 +6672,7 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="28" t="inlineStr">
+      <c r="A17" s="30" t="inlineStr">
         <is>
           <t>caller_rel_height</t>
         </is>
@@ -6437,7 +6687,7 @@
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="28" t="inlineStr">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>edge_guard_s</t>
         </is>
@@ -6452,7 +6702,7 @@
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A19" s="30" t="inlineStr">
         <is>
           <t>chunk_duration_s</t>
         </is>
@@ -6467,7 +6717,7 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="28" t="inlineStr">
+      <c r="A20" s="30" t="inlineStr">
         <is>
           <t>chunk_overlap_s</t>
         </is>
@@ -6482,7 +6732,7 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="28" t="inlineStr">
+      <c r="A21" s="30" t="inlineStr">
         <is>
           <t>spectrogram_preview_s</t>
         </is>
@@ -6492,7 +6742,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>PNG só da primeira janela; este lote usou --no-spectrogram.</t>
+          <t>PNG de arquivos longos = janela de 60 s com mais picos, não os primeiros 60 s. Validação da tese: aba Espectrogramas.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tornar gráficos e relatórios mais intuitivos para a tese
- Excel provisório: rótulos de pico nos gráficos, guia das abas, legenda
  em Espectrogramas, colunas Campanhas mais claras (soma vs média)
- resultado.xlsx (report.py): abas e gráficos em português, notas de leitura
- Painel: banner PROVISÓRIO, aviso do teto 1–2, cards com subtítulos,
  gráficos hora/mês com caveats e destaque do pico, tabelas com tooltips

Co-authored-by: Antonio Junior <antoniocfjr@icloud.com>
</commit_message>
<xml_diff>
--- a/reports/relatorio_provisorio.xlsx
+++ b/reports/relatorio_provisorio.xlsx
@@ -30,7 +30,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,11 +66,17 @@
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002F5D50"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <name val="Consolas"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -112,6 +118,11 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E4EEE9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -139,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -213,17 +224,20 @@
     <xf numFmtId="3" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -337,10 +351,17 @@
             </strRef>
           </tx>
           <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2F5D50"/>
+            </a:solidFill>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <showVal val="1"/>
+          </dLbls>
           <cat>
             <numRef>
               <f>'Por hora'!$A$4:$A$27</f>
@@ -448,10 +469,17 @@
             </strRef>
           </tx>
           <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2F5D50"/>
+            </a:solidFill>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <showVal val="1"/>
+          </dLbls>
           <cat>
             <numRef>
               <f>'Por mês'!$A$4:$A$15</f>
@@ -587,7 +615,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>9</row>
+      <row>10</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6096000" cy="3267075"/>
@@ -612,7 +640,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>12</row>
+      <row>13</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6096000" cy="3267075"/>
@@ -637,7 +665,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>15</row>
+      <row>16</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6096000" cy="3267075"/>
@@ -951,7 +979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -981,84 +1009,96 @@
     <row r="3" ht="78" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Guia das abas</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Este livro é PROVISÓRIO: serve para a aluna abrir, enviar por e-mail e usar no rascunho da tese. Não substitui a lista completa de eventos (output/resultado.xlsx, ~7 MB, gitignored). A aba Espectrogramas traz o recorte de escuta da madrugada com os picos marcados (validação humana). Não há um PNG por evento do lote (isso seriam ~150 mil imagens).</t>
+          <t>Leia primeiro (este texto) · Resumo (totais) · Campanhas (por pasta) · Arquivos (por gravação) · Por hora / Por mês (início do arquivo) · Ouvir (recorte 30:45 para validação) · Espectrogramas (PNG da madrugada) · Parâmetros (DetectionConfig, só leitura).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="78" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>O que os números são</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Contagem automática de eventos acústicos — picos de energia na banda calibrada 2,6–3,2 kHz (referência Áudio base/CEAES 2.m4a, pico ~2,89 kHz). Mesmo DetectionConfig em 75 arquivos, 104.742 h, 149962 eventos, 0 erros de processamento. Pipeline gerado em 2026-09-01T13:20:58.828375+00:00.</t>
+          <t>Este livro é PROVISÓRIO: serve para a aluna abrir, enviar por e-mail e usar no rascunho da tese. Não substitui a lista completa de eventos (output/resultado.xlsx, ~7 MB, gitignored). A aba Espectrogramas traz o recorte de escuta da madrugada com os picos marcados (validação humana). Não há um PNG por evento do lote (isso seriam ~150 mil imagens).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="78" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>O que NÃO afirmar</t>
+          <t>O que os números são</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Não são 149 962 machos, indivíduos ou pererecas. Um macho gera muitos eventos; dois machos no mesmo pitch podem virar um. Qualquer energia na banda acima do limiar vira evento (inseto, gravador, outra espécie). Não se comprovou espécie até de manhã. max_simultaneous = 2 é teto estrutural da banda de 600 Hz com separação de 400 Hz, não um censo. A Fase 3 (Claude) não foi usada.</t>
+          <t>Contagem automática de eventos acústicos — picos de energia na banda calibrada 2,6–3,2 kHz (referência Áudio base/CEAES 2.m4a, pico ~2,89 kHz). Mesmo DetectionConfig em 75 arquivos, 104.742 h, 149962 eventos, 0 erros de processamento. Pipeline gerado em 2026-09-01T13:20:58.828375+00:00.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="78" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Gráficos hora / mês</t>
+          <t>O que NÃO afirmar</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>A hora/mês é a do INÍCIO do arquivo (nome RYYYYMMDD-HHMMSS), não o relógio de cada canto. Sete MP3s (campanhas 12_09_25 e 15_08_25) não têm data no nome: 50 170 eventos entram no total e saem dos gráficos. Zeros às 11–13 h = nenhum WAV a começar nessa hora, não «zero canto». Agosto/setembro vazios nos gráficos pelas mesmas MP3s.</t>
+          <t>Não são 149 962 machos, indivíduos ou pererecas. Um macho gera muitos eventos; dois machos no mesmo pitch podem virar um. Qualquer energia na banda acima do limiar vira evento (inseto, gravador, outra espécie). Não se comprovou espécie até de manhã. max_simultaneous = 2 é teto estrutural da banda de 600 Hz com separação de 400 Hz, não um censo. A Fase 3 (Claude) não foi usada.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="78" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Próximo passo</t>
+          <t>Gráficos hora / mês</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Escuta humana do recorte já escolhido (aba Ouvir): pasta «10_10_25 açude 1», ficheiro R20241012-041002.WAV, gravado em 2024-10-12T04:10:02. Seek 30:45 (1845 s), ouvir 60 s até 31:45. Relógio de campo 04:40:47–04:41:47. O detector marcou 64 eventos curtos (~0.1 s), mediana ~2918 Hz (CEAES 2 ~2.89 kHz). Comparar com Áudio base/CEAES 2.m4a. NÃO começar pelo ficheiro da manhã R20241012-091022.WAV (09:10, o mais denso); só depois de o recorte da madrugada soar a rã.</t>
+          <t>A hora/mês é a do INÍCIO do arquivo (nome RYYYYMMDD-HHMMSS), não o relógio de cada canto. Sete MP3s (campanhas 12_09_25 e 15_08_25) não têm data no nome: 50 170 eventos entram no total e saem dos gráficos. Zeros às 11–13 h = nenhum WAV a começar nessa hora, não «zero canto». Agosto/setembro vazios nos gráficos pelas mesmas MP3s.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="78" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Documentos</t>
+          <t>Próximo passo</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>O que a tese pode afirmar: docs/PRECISAO_E_LIMITES.md. Como ler Excel/JSON completos: docs/COMO_LER_OS_RESULTADOS.md. Parâmetros: aba Parâmetros e src/bioacoustics/config.py. Totais enxutos: reports/campo_resumo.json. PNG de validação: aba Espectrogramas e reports/espectrogramas/.</t>
+          <t>Escuta humana do recorte já escolhido (aba Ouvir): pasta «10_10_25 açude 1», ficheiro R20241012-041002.WAV, gravado em 2024-10-12T04:10:02. Seek 30:45 (1845 s), ouvir 60 s até 31:45. Relógio de campo 04:40:47–04:41:47. O detector marcou 64 eventos curtos (~0.1 s), mediana ~2918 Hz (CEAES 2 ~2.89 kHz). Comparar com Áudio base/CEAES 2.m4a. NÃO começar pelo ficheiro da manhã R20241012-091022.WAV (09:10, o mais denso); só depois de o recorte da madrugada soar a rã.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="78" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
+          <t>Documentos</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>O que a tese pode afirmar: docs/PRECISAO_E_LIMITES.md. Como ler Excel/JSON completos: docs/COMO_LER_OS_RESULTADOS.md. Parâmetros: aba Parâmetros e src/bioacoustics/config.py. Totais enxutos: reports/campo_resumo.json. PNG de validação: aba Espectrogramas e reports/espectrogramas/.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="78" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
           <t>Como regenerar</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>python3 scripts/export_relatorio_provisorio.py  (gerado 2026-09-02 13:04 UTC). 64 eventos do recorte listados na aba Ouvir (extraídos de output/resultado.json).</t>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>python3 scripts/export_relatorio_provisorio.py  (gerado 2026-09-02 18:22 UTC). Lista dos 64 eventos do recorte ausente: rode o script na máquina com output/resultado.json para a preencher.</t>
         </is>
       </c>
     </row>
@@ -1393,7 +1433,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Pastas de açude 1. «15/08 açude 2 (esse nao precisa)» e «Áudio base» não entram. Campanhas só com MP3s não têm recorded_at.</t>
+          <t>Pastas de açude 1. «Eventos (soma)» = total de picos na campanha; «Eventos/h (média)» = média por arquivo (não é densidade horária do gráfico). MP3s sem data no nome ficam destacados.</t>
         </is>
       </c>
       <c r="B2" s="7" t="n"/>
@@ -1416,7 +1456,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Eventos</t>
+          <t>Eventos (soma)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1426,7 +1466,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Eventos/h</t>
+          <t>Eventos/h (média)</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -3845,7 +3885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4181,10 +4221,18 @@
       </c>
       <c r="C27" s="9" t="inlineStr"/>
     </row>
+    <row r="29">
+      <c r="A29" s="27" t="inlineStr">
+        <is>
+          <t>Pico: 05h — 7.181 eventos (início de arquivo neste bloco)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A29:F29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4198,7 +4246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4422,10 +4470,18 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>Pico: 10 out — 58.743 eventos (início de arquivo neste bloco)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4439,7 +4495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4634,1610 +4690,10 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B15" s="15" t="n">
-        <v>1845.339</v>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>04:40:47</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="n">
-        <v>3090</v>
-      </c>
-      <c r="E15" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F15" s="15" t="n">
-        <v>28.038</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B16" s="15" t="n">
-        <v>1845.85</v>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>04:40:47</t>
-        </is>
-      </c>
-      <c r="D16" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E16" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F16" s="15" t="n">
-        <v>74.901</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B17" s="15" t="n">
-        <v>1846.384</v>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>04:40:48</t>
-        </is>
-      </c>
-      <c r="D17" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E17" s="15" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="F17" s="15" t="n">
-        <v>42.902</v>
-      </c>
-      <c r="G17" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B18" s="15" t="n">
-        <v>1846.872</v>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>04:40:48</t>
-        </is>
-      </c>
-      <c r="D18" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E18" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F18" s="15" t="n">
-        <v>55.072</v>
-      </c>
-      <c r="G18" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B19" s="15" t="n">
-        <v>1847.452</v>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>04:40:49</t>
-        </is>
-      </c>
-      <c r="D19" s="11" t="n">
-        <v>3090</v>
-      </c>
-      <c r="E19" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F19" s="15" t="n">
-        <v>29.62</v>
-      </c>
-      <c r="G19" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B20" s="15" t="n">
-        <v>1848.009</v>
-      </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>04:40:50</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E20" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F20" s="15" t="n">
-        <v>56.337</v>
-      </c>
-      <c r="G20" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B21" s="15" t="n">
-        <v>1848.543</v>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>04:40:50</t>
-        </is>
-      </c>
-      <c r="D21" s="11" t="n">
-        <v>3143.8</v>
-      </c>
-      <c r="E21" s="15" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="F21" s="15" t="n">
-        <v>20.216</v>
-      </c>
-      <c r="G21" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B22" s="15" t="n">
-        <v>1849.078</v>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>04:40:51</t>
-        </is>
-      </c>
-      <c r="D22" s="11" t="n">
-        <v>2939.3</v>
-      </c>
-      <c r="E22" s="15" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="F22" s="15" t="n">
-        <v>33.363</v>
-      </c>
-      <c r="G22" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B23" s="15" t="n">
-        <v>1850.099</v>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>04:40:52</t>
-        </is>
-      </c>
-      <c r="D23" s="11" t="n">
-        <v>2939.3</v>
-      </c>
-      <c r="E23" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F23" s="15" t="n">
-        <v>41.71</v>
-      </c>
-      <c r="G23" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="B24" s="15" t="n">
-        <v>1850.61</v>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>04:40:52</t>
-        </is>
-      </c>
-      <c r="D24" s="11" t="n">
-        <v>3090</v>
-      </c>
-      <c r="E24" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F24" s="15" t="n">
-        <v>47.426</v>
-      </c>
-      <c r="G24" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="n">
-        <v>11</v>
-      </c>
-      <c r="B25" s="15" t="n">
-        <v>1851.121</v>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>04:40:53</t>
-        </is>
-      </c>
-      <c r="D25" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E25" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F25" s="15" t="n">
-        <v>60.029</v>
-      </c>
-      <c r="G25" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="B26" s="15" t="n">
-        <v>1851.678</v>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>04:40:53</t>
-        </is>
-      </c>
-      <c r="D26" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E26" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F26" s="15" t="n">
-        <v>36.121</v>
-      </c>
-      <c r="G26" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="n">
-        <v>13</v>
-      </c>
-      <c r="B27" s="15" t="n">
-        <v>1852.259</v>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>04:40:54</t>
-        </is>
-      </c>
-      <c r="D27" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E27" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F27" s="15" t="n">
-        <v>62.92</v>
-      </c>
-      <c r="G27" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="9" t="n">
-        <v>14</v>
-      </c>
-      <c r="B28" s="15" t="n">
-        <v>1853.118</v>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>04:40:55</t>
-        </is>
-      </c>
-      <c r="D28" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E28" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F28" s="15" t="n">
-        <v>49.537</v>
-      </c>
-      <c r="G28" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="n">
-        <v>15</v>
-      </c>
-      <c r="B29" s="15" t="n">
-        <v>1853.652</v>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>04:40:55</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E29" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F29" s="15" t="n">
-        <v>90.636</v>
-      </c>
-      <c r="G29" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="9" t="n">
-        <v>16</v>
-      </c>
-      <c r="B30" s="15" t="n">
-        <v>1854.697</v>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>04:40:56</t>
-        </is>
-      </c>
-      <c r="D30" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E30" s="15" t="n">
-        <v>0.302</v>
-      </c>
-      <c r="F30" s="15" t="n">
-        <v>83.167</v>
-      </c>
-      <c r="G30" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="n">
-        <v>17</v>
-      </c>
-      <c r="B31" s="15" t="n">
-        <v>1855.44</v>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>04:40:57</t>
-        </is>
-      </c>
-      <c r="D31" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E31" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F31" s="15" t="n">
-        <v>89.595</v>
-      </c>
-      <c r="G31" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="9" t="n">
-        <v>18</v>
-      </c>
-      <c r="B32" s="15" t="n">
-        <v>1855.951</v>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>04:40:57</t>
-        </is>
-      </c>
-      <c r="D32" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E32" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F32" s="15" t="n">
-        <v>32.234</v>
-      </c>
-      <c r="G32" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="9" t="n">
-        <v>19</v>
-      </c>
-      <c r="B33" s="15" t="n">
-        <v>1856.67</v>
-      </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>04:40:58</t>
-        </is>
-      </c>
-      <c r="D33" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E33" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F33" s="15" t="n">
-        <v>69.297</v>
-      </c>
-      <c r="G33" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="B34" s="15" t="n">
-        <v>1857.762</v>
-      </c>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t>04:40:59</t>
-        </is>
-      </c>
-      <c r="D34" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E34" s="15" t="n">
-        <v>1.207</v>
-      </c>
-      <c r="F34" s="15" t="n">
-        <v>75.598</v>
-      </c>
-      <c r="G34" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="9" t="n">
-        <v>21</v>
-      </c>
-      <c r="B35" s="15" t="n">
-        <v>1860.084</v>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>04:41:02</t>
-        </is>
-      </c>
-      <c r="D35" s="11" t="n">
-        <v>2799.3</v>
-      </c>
-      <c r="E35" s="15" t="n">
-        <v>0.929</v>
-      </c>
-      <c r="F35" s="15" t="n">
-        <v>12.49</v>
-      </c>
-      <c r="G35" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="B36" s="15" t="n">
-        <v>1861.802</v>
-      </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>04:41:03</t>
-        </is>
-      </c>
-      <c r="D36" s="11" t="n">
-        <v>2605.5</v>
-      </c>
-      <c r="E36" s="15" t="n">
-        <v>0.255</v>
-      </c>
-      <c r="F36" s="15" t="n">
-        <v>7.557</v>
-      </c>
-      <c r="G36" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="9" t="n">
-        <v>23</v>
-      </c>
-      <c r="B37" s="15" t="n">
-        <v>1863.335</v>
-      </c>
-      <c r="C37" s="9" t="inlineStr">
-        <is>
-          <t>04:41:05</t>
-        </is>
-      </c>
-      <c r="D37" s="11" t="n">
-        <v>2637.8</v>
-      </c>
-      <c r="E37" s="15" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="F37" s="15" t="n">
-        <v>18.349</v>
-      </c>
-      <c r="G37" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="9" t="n">
-        <v>24</v>
-      </c>
-      <c r="B38" s="15" t="n">
-        <v>1864.054</v>
-      </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>04:41:06</t>
-        </is>
-      </c>
-      <c r="D38" s="11" t="n">
-        <v>2745.5</v>
-      </c>
-      <c r="E38" s="15" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="F38" s="15" t="n">
-        <v>13.575</v>
-      </c>
-      <c r="G38" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="9" t="n">
-        <v>25</v>
-      </c>
-      <c r="B39" s="15" t="n">
-        <v>1865.262</v>
-      </c>
-      <c r="C39" s="9" t="inlineStr">
-        <is>
-          <t>04:41:07</t>
-        </is>
-      </c>
-      <c r="D39" s="11" t="n">
-        <v>2788.5</v>
-      </c>
-      <c r="E39" s="15" t="n">
-        <v>0.163</v>
-      </c>
-      <c r="F39" s="15" t="n">
-        <v>14.993</v>
-      </c>
-      <c r="G39" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="B40" s="15" t="n">
-        <v>1866.214</v>
-      </c>
-      <c r="C40" s="9" t="inlineStr">
-        <is>
-          <t>04:41:08</t>
-        </is>
-      </c>
-      <c r="D40" s="11" t="n">
-        <v>2734.7</v>
-      </c>
-      <c r="E40" s="15" t="n">
-        <v>0.139</v>
-      </c>
-      <c r="F40" s="15" t="n">
-        <v>12.565</v>
-      </c>
-      <c r="G40" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="9" t="n">
-        <v>27</v>
-      </c>
-      <c r="B41" s="15" t="n">
-        <v>1870.115</v>
-      </c>
-      <c r="C41" s="9" t="inlineStr">
-        <is>
-          <t>04:41:12</t>
-        </is>
-      </c>
-      <c r="D41" s="11" t="n">
-        <v>2982.3</v>
-      </c>
-      <c r="E41" s="15" t="n">
-        <v>2.02</v>
-      </c>
-      <c r="F41" s="15" t="n">
-        <v>29.627</v>
-      </c>
-      <c r="G41" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="9" t="n">
-        <v>28</v>
-      </c>
-      <c r="B42" s="15" t="n">
-        <v>1870.788</v>
-      </c>
-      <c r="C42" s="9" t="inlineStr">
-        <is>
-          <t>04:41:12</t>
-        </is>
-      </c>
-      <c r="D42" s="11" t="n">
-        <v>2637.8</v>
-      </c>
-      <c r="E42" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F42" s="15" t="n">
-        <v>16.208</v>
-      </c>
-      <c r="G42" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="9" t="n">
-        <v>29</v>
-      </c>
-      <c r="B43" s="15" t="n">
-        <v>1871.276</v>
-      </c>
-      <c r="C43" s="9" t="inlineStr">
-        <is>
-          <t>04:41:13</t>
-        </is>
-      </c>
-      <c r="D43" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E43" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F43" s="15" t="n">
-        <v>29.953</v>
-      </c>
-      <c r="G43" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="B44" s="15" t="n">
-        <v>1872.274</v>
-      </c>
-      <c r="C44" s="9" t="inlineStr">
-        <is>
-          <t>04:41:14</t>
-        </is>
-      </c>
-      <c r="D44" s="11" t="n">
-        <v>2960.8</v>
-      </c>
-      <c r="E44" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F44" s="15" t="n">
-        <v>31.616</v>
-      </c>
-      <c r="G44" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="9" t="n">
-        <v>31</v>
-      </c>
-      <c r="B45" s="15" t="n">
-        <v>1872.785</v>
-      </c>
-      <c r="C45" s="9" t="inlineStr">
-        <is>
-          <t>04:41:14</t>
-        </is>
-      </c>
-      <c r="D45" s="11" t="n">
-        <v>3165.4</v>
-      </c>
-      <c r="E45" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F45" s="15" t="n">
-        <v>14.018</v>
-      </c>
-      <c r="G45" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="9" t="n">
-        <v>32</v>
-      </c>
-      <c r="B46" s="15" t="n">
-        <v>1873.296</v>
-      </c>
-      <c r="C46" s="9" t="inlineStr">
-        <is>
-          <t>04:41:15</t>
-        </is>
-      </c>
-      <c r="D46" s="11" t="n">
-        <v>2799.3</v>
-      </c>
-      <c r="E46" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F46" s="15" t="n">
-        <v>30.776</v>
-      </c>
-      <c r="G46" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="9" t="n">
-        <v>33</v>
-      </c>
-      <c r="B47" s="15" t="n">
-        <v>1874.294</v>
-      </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>04:41:16</t>
-        </is>
-      </c>
-      <c r="D47" s="11" t="n">
-        <v>2820.8</v>
-      </c>
-      <c r="E47" s="15" t="n">
-        <v>0.604</v>
-      </c>
-      <c r="F47" s="15" t="n">
-        <v>37.613</v>
-      </c>
-      <c r="G47" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="9" t="n">
-        <v>34</v>
-      </c>
-      <c r="B48" s="15" t="n">
-        <v>1875.293</v>
-      </c>
-      <c r="C48" s="9" t="inlineStr">
-        <is>
-          <t>04:41:17</t>
-        </is>
-      </c>
-      <c r="D48" s="11" t="n">
-        <v>2702.4</v>
-      </c>
-      <c r="E48" s="15" t="n">
-        <v>0.139</v>
-      </c>
-      <c r="F48" s="15" t="n">
-        <v>30.969</v>
-      </c>
-      <c r="G48" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="9" t="n">
-        <v>35</v>
-      </c>
-      <c r="B49" s="15" t="n">
-        <v>1875.827</v>
-      </c>
-      <c r="C49" s="9" t="inlineStr">
-        <is>
-          <t>04:41:17</t>
-        </is>
-      </c>
-      <c r="D49" s="11" t="n">
-        <v>3176.1</v>
-      </c>
-      <c r="E49" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F49" s="15" t="n">
-        <v>17.356</v>
-      </c>
-      <c r="G49" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="9" t="n">
-        <v>36</v>
-      </c>
-      <c r="B50" s="15" t="n">
-        <v>1876.616</v>
-      </c>
-      <c r="C50" s="9" t="inlineStr">
-        <is>
-          <t>04:41:18</t>
-        </is>
-      </c>
-      <c r="D50" s="11" t="n">
-        <v>2788.5</v>
-      </c>
-      <c r="E50" s="15" t="n">
-        <v>0.232</v>
-      </c>
-      <c r="F50" s="15" t="n">
-        <v>42.013</v>
-      </c>
-      <c r="G50" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="9" t="n">
-        <v>37</v>
-      </c>
-      <c r="B51" s="15" t="n">
-        <v>1877.359</v>
-      </c>
-      <c r="C51" s="9" t="inlineStr">
-        <is>
-          <t>04:41:19</t>
-        </is>
-      </c>
-      <c r="D51" s="11" t="n">
-        <v>3079.2</v>
-      </c>
-      <c r="E51" s="15" t="n">
-        <v>0.325</v>
-      </c>
-      <c r="F51" s="15" t="n">
-        <v>10.056</v>
-      </c>
-      <c r="G51" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="9" t="n">
-        <v>38</v>
-      </c>
-      <c r="B52" s="15" t="n">
-        <v>1877.824</v>
-      </c>
-      <c r="C52" s="9" t="inlineStr">
-        <is>
-          <t>04:41:19</t>
-        </is>
-      </c>
-      <c r="D52" s="11" t="n">
-        <v>2724</v>
-      </c>
-      <c r="E52" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F52" s="15" t="n">
-        <v>27.472</v>
-      </c>
-      <c r="G52" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="9" t="n">
-        <v>39</v>
-      </c>
-      <c r="B53" s="15" t="n">
-        <v>1878.846</v>
-      </c>
-      <c r="C53" s="9" t="inlineStr">
-        <is>
-          <t>04:41:20</t>
-        </is>
-      </c>
-      <c r="D53" s="11" t="n">
-        <v>2917.7</v>
-      </c>
-      <c r="E53" s="15" t="n">
-        <v>0.5570000000000001</v>
-      </c>
-      <c r="F53" s="15" t="n">
-        <v>28.289</v>
-      </c>
-      <c r="G53" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="9" t="n">
-        <v>40</v>
-      </c>
-      <c r="B54" s="15" t="n">
-        <v>1879.356</v>
-      </c>
-      <c r="C54" s="9" t="inlineStr">
-        <is>
-          <t>04:41:21</t>
-        </is>
-      </c>
-      <c r="D54" s="11" t="n">
-        <v>2971.6</v>
-      </c>
-      <c r="E54" s="15" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="F54" s="15" t="n">
-        <v>27.926</v>
-      </c>
-      <c r="G54" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="9" t="n">
-        <v>41</v>
-      </c>
-      <c r="B55" s="15" t="n">
-        <v>1881.051</v>
-      </c>
-      <c r="C55" s="9" t="inlineStr">
-        <is>
-          <t>04:41:23</t>
-        </is>
-      </c>
-      <c r="D55" s="11" t="n">
-        <v>2767</v>
-      </c>
-      <c r="E55" s="15" t="n">
-        <v>1.463</v>
-      </c>
-      <c r="F55" s="15" t="n">
-        <v>35.758</v>
-      </c>
-      <c r="G55" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="9" t="n">
-        <v>42</v>
-      </c>
-      <c r="B56" s="15" t="n">
-        <v>1882.375</v>
-      </c>
-      <c r="C56" s="9" t="inlineStr">
-        <is>
-          <t>04:41:24</t>
-        </is>
-      </c>
-      <c r="D56" s="11" t="n">
-        <v>2777.8</v>
-      </c>
-      <c r="E56" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F56" s="15" t="n">
-        <v>32.074</v>
-      </c>
-      <c r="G56" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="9" t="n">
-        <v>43</v>
-      </c>
-      <c r="B57" s="15" t="n">
-        <v>1882.95</v>
-      </c>
-      <c r="C57" s="9" t="inlineStr">
-        <is>
-          <t>04:41:24</t>
-        </is>
-      </c>
-      <c r="D57" s="11" t="n">
-        <v>2724</v>
-      </c>
-      <c r="E57" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F57" s="15" t="n">
-        <v>23.89</v>
-      </c>
-      <c r="G57" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="9" t="n">
-        <v>44</v>
-      </c>
-      <c r="B58" s="15" t="n">
-        <v>1883.461</v>
-      </c>
-      <c r="C58" s="9" t="inlineStr">
-        <is>
-          <t>04:41:25</t>
-        </is>
-      </c>
-      <c r="D58" s="11" t="n">
-        <v>2767</v>
-      </c>
-      <c r="E58" s="15" t="n">
-        <v>0.186</v>
-      </c>
-      <c r="F58" s="15" t="n">
-        <v>33.822</v>
-      </c>
-      <c r="G58" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="9" t="n">
-        <v>45</v>
-      </c>
-      <c r="B59" s="15" t="n">
-        <v>1884.576</v>
-      </c>
-      <c r="C59" s="9" t="inlineStr">
-        <is>
-          <t>04:41:26</t>
-        </is>
-      </c>
-      <c r="D59" s="11" t="n">
-        <v>3046.9</v>
-      </c>
-      <c r="E59" s="15" t="n">
-        <v>0.186</v>
-      </c>
-      <c r="F59" s="15" t="n">
-        <v>16.543</v>
-      </c>
-      <c r="G59" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="9" t="n">
-        <v>46</v>
-      </c>
-      <c r="B60" s="15" t="n">
-        <v>1885.83</v>
-      </c>
-      <c r="C60" s="9" t="inlineStr">
-        <is>
-          <t>04:41:27</t>
-        </is>
-      </c>
-      <c r="D60" s="11" t="n">
-        <v>2874.7</v>
-      </c>
-      <c r="E60" s="15" t="n">
-        <v>1.277</v>
-      </c>
-      <c r="F60" s="15" t="n">
-        <v>24.839</v>
-      </c>
-      <c r="G60" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="9" t="n">
-        <v>47</v>
-      </c>
-      <c r="B61" s="15" t="n">
-        <v>1887.014</v>
-      </c>
-      <c r="C61" s="9" t="inlineStr">
-        <is>
-          <t>04:41:29</t>
-        </is>
-      </c>
-      <c r="D61" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E61" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F61" s="15" t="n">
-        <v>24.112</v>
-      </c>
-      <c r="G61" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="9" t="n">
-        <v>48</v>
-      </c>
-      <c r="B62" s="15" t="n">
-        <v>1888.152</v>
-      </c>
-      <c r="C62" s="9" t="inlineStr">
-        <is>
-          <t>04:41:30</t>
-        </is>
-      </c>
-      <c r="D62" s="11" t="n">
-        <v>2745.5</v>
-      </c>
-      <c r="E62" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F62" s="15" t="n">
-        <v>17.237</v>
-      </c>
-      <c r="G62" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="9" t="n">
-        <v>49</v>
-      </c>
-      <c r="B63" s="15" t="n">
-        <v>1888.732</v>
-      </c>
-      <c r="C63" s="9" t="inlineStr">
-        <is>
-          <t>04:41:30</t>
-        </is>
-      </c>
-      <c r="D63" s="11" t="n">
-        <v>2713.2</v>
-      </c>
-      <c r="E63" s="15" t="n">
-        <v>0.998</v>
-      </c>
-      <c r="F63" s="15" t="n">
-        <v>21.434</v>
-      </c>
-      <c r="G63" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="9" t="n">
-        <v>50</v>
-      </c>
-      <c r="B64" s="15" t="n">
-        <v>1890.66</v>
-      </c>
-      <c r="C64" s="9" t="inlineStr">
-        <is>
-          <t>04:41:32</t>
-        </is>
-      </c>
-      <c r="D64" s="11" t="n">
-        <v>2799.3</v>
-      </c>
-      <c r="E64" s="15" t="n">
-        <v>0.604</v>
-      </c>
-      <c r="F64" s="15" t="n">
-        <v>29.823</v>
-      </c>
-      <c r="G64" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="9" t="n">
-        <v>51</v>
-      </c>
-      <c r="B65" s="15" t="n">
-        <v>1891.728</v>
-      </c>
-      <c r="C65" s="9" t="inlineStr">
-        <is>
-          <t>04:41:33</t>
-        </is>
-      </c>
-      <c r="D65" s="11" t="n">
-        <v>2767</v>
-      </c>
-      <c r="E65" s="15" t="n">
-        <v>0.604</v>
-      </c>
-      <c r="F65" s="15" t="n">
-        <v>22.563</v>
-      </c>
-      <c r="G65" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="9" t="n">
-        <v>52</v>
-      </c>
-      <c r="B66" s="15" t="n">
-        <v>1892.796</v>
-      </c>
-      <c r="C66" s="9" t="inlineStr">
-        <is>
-          <t>04:41:34</t>
-        </is>
-      </c>
-      <c r="D66" s="11" t="n">
-        <v>2777.8</v>
-      </c>
-      <c r="E66" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F66" s="15" t="n">
-        <v>37.032</v>
-      </c>
-      <c r="G66" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="9" t="n">
-        <v>53</v>
-      </c>
-      <c r="B67" s="15" t="n">
-        <v>1893.817</v>
-      </c>
-      <c r="C67" s="9" t="inlineStr">
-        <is>
-          <t>04:41:35</t>
-        </is>
-      </c>
-      <c r="D67" s="11" t="n">
-        <v>2756.2</v>
-      </c>
-      <c r="E67" s="15" t="n">
-        <v>0.604</v>
-      </c>
-      <c r="F67" s="15" t="n">
-        <v>39.972</v>
-      </c>
-      <c r="G67" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="9" t="n">
-        <v>54</v>
-      </c>
-      <c r="B68" s="15" t="n">
-        <v>1894.886</v>
-      </c>
-      <c r="C68" s="9" t="inlineStr">
-        <is>
-          <t>04:41:36</t>
-        </is>
-      </c>
-      <c r="D68" s="11" t="n">
-        <v>2767</v>
-      </c>
-      <c r="E68" s="15" t="n">
-        <v>0.163</v>
-      </c>
-      <c r="F68" s="15" t="n">
-        <v>31.216</v>
-      </c>
-      <c r="G68" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="9" t="n">
-        <v>55</v>
-      </c>
-      <c r="B69" s="15" t="n">
-        <v>1895.443</v>
-      </c>
-      <c r="C69" s="9" t="inlineStr">
-        <is>
-          <t>04:41:37</t>
-        </is>
-      </c>
-      <c r="D69" s="11" t="n">
-        <v>3068.5</v>
-      </c>
-      <c r="E69" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F69" s="15" t="n">
-        <v>39.844</v>
-      </c>
-      <c r="G69" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="9" t="n">
-        <v>56</v>
-      </c>
-      <c r="B70" s="15" t="n">
-        <v>1895.977</v>
-      </c>
-      <c r="C70" s="9" t="inlineStr">
-        <is>
-          <t>04:41:37</t>
-        </is>
-      </c>
-      <c r="D70" s="11" t="n">
-        <v>2713.2</v>
-      </c>
-      <c r="E70" s="15" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="F70" s="15" t="n">
-        <v>29.673</v>
-      </c>
-      <c r="G70" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="9" t="n">
-        <v>57</v>
-      </c>
-      <c r="B71" s="15" t="n">
-        <v>1896.488</v>
-      </c>
-      <c r="C71" s="9" t="inlineStr">
-        <is>
-          <t>04:41:38</t>
-        </is>
-      </c>
-      <c r="D71" s="11" t="n">
-        <v>2767</v>
-      </c>
-      <c r="E71" s="15" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="F71" s="15" t="n">
-        <v>22.536</v>
-      </c>
-      <c r="G71" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="9" t="n">
-        <v>58</v>
-      </c>
-      <c r="B72" s="15" t="n">
-        <v>1898.02</v>
-      </c>
-      <c r="C72" s="9" t="inlineStr">
-        <is>
-          <t>04:41:40</t>
-        </is>
-      </c>
-      <c r="D72" s="11" t="n">
-        <v>2831.6</v>
-      </c>
-      <c r="E72" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F72" s="15" t="n">
-        <v>18.32</v>
-      </c>
-      <c r="G72" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="9" t="n">
-        <v>59</v>
-      </c>
-      <c r="B73" s="15" t="n">
-        <v>1898.903</v>
-      </c>
-      <c r="C73" s="9" t="inlineStr">
-        <is>
-          <t>04:41:40</t>
-        </is>
-      </c>
-      <c r="D73" s="11" t="n">
-        <v>2745.5</v>
-      </c>
-      <c r="E73" s="15" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="F73" s="15" t="n">
-        <v>13.27</v>
-      </c>
-      <c r="G73" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="9" t="n">
-        <v>60</v>
-      </c>
-      <c r="B74" s="15" t="n">
-        <v>1899.53</v>
-      </c>
-      <c r="C74" s="9" t="inlineStr">
-        <is>
-          <t>04:41:41</t>
-        </is>
-      </c>
-      <c r="D74" s="11" t="n">
-        <v>2745.5</v>
-      </c>
-      <c r="E74" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F74" s="15" t="n">
-        <v>12.409</v>
-      </c>
-      <c r="G74" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="9" t="n">
-        <v>61</v>
-      </c>
-      <c r="B75" s="15" t="n">
-        <v>1900.528</v>
-      </c>
-      <c r="C75" s="9" t="inlineStr">
-        <is>
-          <t>04:41:42</t>
-        </is>
-      </c>
-      <c r="D75" s="11" t="n">
-        <v>2745.5</v>
-      </c>
-      <c r="E75" s="15" t="n">
-        <v>0.209</v>
-      </c>
-      <c r="F75" s="15" t="n">
-        <v>41.317</v>
-      </c>
-      <c r="G75" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="9" t="n">
-        <v>62</v>
-      </c>
-      <c r="B76" s="15" t="n">
-        <v>1902.618</v>
-      </c>
-      <c r="C76" s="9" t="inlineStr">
-        <is>
-          <t>04:41:44</t>
-        </is>
-      </c>
-      <c r="D76" s="11" t="n">
-        <v>2767</v>
-      </c>
-      <c r="E76" s="15" t="n">
-        <v>1.138</v>
-      </c>
-      <c r="F76" s="15" t="n">
-        <v>39.177</v>
-      </c>
-      <c r="G76" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="9" t="n">
-        <v>63</v>
-      </c>
-      <c r="B77" s="15" t="n">
-        <v>1903.129</v>
-      </c>
-      <c r="C77" s="9" t="inlineStr">
-        <is>
-          <t>04:41:45</t>
-        </is>
-      </c>
-      <c r="D77" s="11" t="n">
-        <v>3090</v>
-      </c>
-      <c r="E77" s="15" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="F77" s="15" t="n">
-        <v>18.748</v>
-      </c>
-      <c r="G77" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="9" t="n">
-        <v>64</v>
-      </c>
-      <c r="B78" s="15" t="n">
-        <v>1904.684</v>
-      </c>
-      <c r="C78" s="9" t="inlineStr">
-        <is>
-          <t>04:41:46</t>
-        </is>
-      </c>
-      <c r="D78" s="11" t="n">
-        <v>2767</v>
-      </c>
-      <c r="E78" s="15" t="n">
-        <v>1.393</v>
-      </c>
-      <c r="F78" s="15" t="n">
-        <v>35.251</v>
-      </c>
-      <c r="G78" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="27" t="inlineStr">
-        <is>
-          <t>64 eventos no recorte 30:45–31:45 (ficheiro R20241012-041002.WAV). Duração mediana 0.116 s; frequência mediana 2917.7 Hz.</t>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>Lista dos 64 eventos indisponível neste ficheiro: output/resultado.json não estava presente (CI / máquina sem o JSON completo). Na cópia da tese gerada com o JSON local, esta tabela tem uma linha por evento (peak_time_s, relógio, frequência, duração, energia, n_callers). O recorte em si não muda.</t>
         </is>
       </c>
     </row>
@@ -6247,12 +4703,12 @@
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B5:G5"/>
-    <mergeCell ref="A79:G79"/>
     <mergeCell ref="B9:G9"/>
     <mergeCell ref="B8:G8"/>
     <mergeCell ref="B4:G4"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="B12:G12"/>
+    <mergeCell ref="A15:G15"/>
     <mergeCell ref="B7:G7"/>
     <mergeCell ref="B11:G11"/>
     <mergeCell ref="B6:G6"/>
@@ -6268,7 +4724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6297,55 +4753,42 @@
       <c r="C2" s="7" t="n"/>
       <c r="D2" s="7" t="n"/>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3" ht="36" customHeight="1">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>Como ler: fundo escuro = espectrograma; linha/círculo verde = pico do detector naquele instante (não re-detecção visual); eixo horizontal = tempo; vertical = kHz. Serve para ouvir+ver se o som parece o anúncio da espécie — não prova ID sozinho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Figura</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Ficheiro</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Legenda</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>reports/espectrogramas/R20241012-041002_30m45s.png</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>embutida</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>R20241012-041002.WAV — 30:45–31:45 (04:40) — picos de vocalização. Recorte de escuta já combinado (64 eventos, ~2,93 kHz). Círculos verdes = eventos do lote, não uma recontagem.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>reports/espectrogramas/R20241012-041002_pico_1854s.png</t>
+          <t>reports/espectrogramas/R20241012-041002_30m45s.png</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -6355,69 +4798,90 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Zoom ~8 s no pico mais forte deste minuto (~1853,65 s, 2928 Hz). Só para conferir a forma do canto; o método de contagem continua a ser a matriz numérica da STFT.</t>
+          <t>R20241012-041002.WAV — 30:45–31:45 (04:40) — picos de vocalização. Recorte de escuta já combinado (64 eventos, ~2,93 kHz). Círculos verdes = eventos do lote, não uma recontagem.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>reports/espectrogramas/R20241012-041002_pico_1854s.png</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>embutida</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Zoom ~8 s no pico mais forte deste minuto (~1853,65 s, 2928 Hz). Só para conferir a forma do canto; o método de contagem continua a ser a matriz numérica da STFT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>reports/espectrogramas/R20241012-091022_densest_60s.png</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>embutida</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>R20241012-091022.WAV — janela de 60 s mais densa — só depois da madrugada. Não começar a validação por este ficheiro.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="28" t="inlineStr">
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>Regenerar PNGs (máquina com o WAV de campo e output/resultado.json): python3 scripts/export_espectrogramas_validacao.py  depois  python3 scripts/export_relatorio_provisorio.py</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="29" t="inlineStr">
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
         <is>
           <t>R20241012-041002.WAV — 30:45–31:45 (04:40) — picos de vocalização. Recorte de escuta já combinado (64 eventos, ~2,93 kHz). Círculos verdes = eventos do lote, não uma recontagem.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="267" customHeight="1"/>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="29" t="inlineStr">
+    <row r="11" ht="267" customHeight="1"/>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="30" t="inlineStr">
         <is>
           <t>Zoom ~8 s no pico mais forte deste minuto (~1853,65 s, 2928 Hz). Só para conferir a forma do canto; o método de contagem continua a ser a matriz numérica da STFT.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="267" customHeight="1"/>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="29" t="inlineStr">
+    <row r="14" ht="267" customHeight="1"/>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>R20241012-091022.WAV — janela de 60 s mais densa — só depois da madrugada. Não começar a validação por este ficheiro.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="267" customHeight="1"/>
+    <row r="17" ht="267" customHeight="1"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A3:D3"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A13:D13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6475,7 +4939,7 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" s="31" t="inlineStr">
         <is>
           <t>sample_rate</t>
         </is>
@@ -6490,7 +4954,7 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="31" t="inlineStr">
         <is>
           <t>lowcut_hz</t>
         </is>
@@ -6505,7 +4969,7 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="A6" s="31" t="inlineStr">
         <is>
           <t>highcut_hz</t>
         </is>
@@ -6520,7 +4984,7 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="30" t="inlineStr">
+      <c r="A7" s="31" t="inlineStr">
         <is>
           <t>filter_order</t>
         </is>
@@ -6535,7 +4999,7 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="30" t="inlineStr">
+      <c r="A8" s="31" t="inlineStr">
         <is>
           <t>n_fft</t>
         </is>
@@ -6550,7 +5014,7 @@
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>hop_length</t>
         </is>
@@ -6565,7 +5029,7 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>use_noise_reduction</t>
         </is>
@@ -6582,7 +5046,7 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>noise_reduce_prop_decrease</t>
         </is>
@@ -6597,7 +5061,7 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>threshold_k</t>
         </is>
@@ -6612,7 +5076,7 @@
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="32" t="inlineStr">
         <is>
           <t>min_peak_distance_s</t>
         </is>
@@ -6620,14 +5084,14 @@
       <c r="B13" s="16" t="n">
         <v>0.15</v>
       </c>
-      <c r="C13" s="32" t="inlineStr">
+      <c r="C13" s="33" t="inlineStr">
         <is>
           <t>Declarado em DetectionConfig; NÃO é usado em detect_events.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>event_merge_gap_s</t>
         </is>
@@ -6642,7 +5106,7 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="30" t="inlineStr">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>min_event_duration_s</t>
         </is>
@@ -6657,7 +5121,7 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="30" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>freq_separation_hz</t>
         </is>
@@ -6672,7 +5136,7 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="30" t="inlineStr">
+      <c r="A17" s="31" t="inlineStr">
         <is>
           <t>caller_rel_height</t>
         </is>
@@ -6687,7 +5151,7 @@
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="30" t="inlineStr">
+      <c r="A18" s="31" t="inlineStr">
         <is>
           <t>edge_guard_s</t>
         </is>
@@ -6702,7 +5166,7 @@
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="30" t="inlineStr">
+      <c r="A19" s="31" t="inlineStr">
         <is>
           <t>chunk_duration_s</t>
         </is>
@@ -6717,7 +5181,7 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="30" t="inlineStr">
+      <c r="A20" s="31" t="inlineStr">
         <is>
           <t>chunk_overlap_s</t>
         </is>
@@ -6732,7 +5196,7 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="30" t="inlineStr">
+      <c r="A21" s="31" t="inlineStr">
         <is>
           <t>spectrogram_preview_s</t>
         </is>

</xml_diff>

<commit_message>
Tornar gráficos e relatórios mais intuitivos para a tese (#12)
- Excel provisório: rótulos de pico nos gráficos, guia das abas, legenda
  em Espectrogramas, colunas Campanhas mais claras (soma vs média)
- resultado.xlsx (report.py): abas e gráficos em português, notas de leitura
- Painel: banner PROVISÓRIO, aviso do teto 1–2, cards com subtítulos,
  gráficos hora/mês com caveats e destaque do pico, tabelas com tooltips

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/reports/relatorio_provisorio.xlsx
+++ b/reports/relatorio_provisorio.xlsx
@@ -30,7 +30,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,11 +66,17 @@
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002F5D50"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <name val="Consolas"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -112,6 +118,11 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E4EEE9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -139,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -213,17 +224,20 @@
     <xf numFmtId="3" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -337,10 +351,17 @@
             </strRef>
           </tx>
           <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2F5D50"/>
+            </a:solidFill>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <showVal val="1"/>
+          </dLbls>
           <cat>
             <numRef>
               <f>'Por hora'!$A$4:$A$27</f>
@@ -448,10 +469,17 @@
             </strRef>
           </tx>
           <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2F5D50"/>
+            </a:solidFill>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <showVal val="1"/>
+          </dLbls>
           <cat>
             <numRef>
               <f>'Por mês'!$A$4:$A$15</f>
@@ -587,7 +615,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>9</row>
+      <row>10</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6096000" cy="3267075"/>
@@ -612,7 +640,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>12</row>
+      <row>13</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6096000" cy="3267075"/>
@@ -637,7 +665,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>15</row>
+      <row>16</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6096000" cy="3267075"/>
@@ -951,7 +979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -981,84 +1009,96 @@
     <row r="3" ht="78" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Guia das abas</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Este livro é PROVISÓRIO: serve para a aluna abrir, enviar por e-mail e usar no rascunho da tese. Não substitui a lista completa de eventos (output/resultado.xlsx, ~7 MB, gitignored). A aba Espectrogramas traz o recorte de escuta da madrugada com os picos marcados (validação humana). Não há um PNG por evento do lote (isso seriam ~150 mil imagens).</t>
+          <t>Leia primeiro (este texto) · Resumo (totais) · Campanhas (por pasta) · Arquivos (por gravação) · Por hora / Por mês (início do arquivo) · Ouvir (recorte 30:45 para validação) · Espectrogramas (PNG da madrugada) · Parâmetros (DetectionConfig, só leitura).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="78" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>O que os números são</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Contagem automática de eventos acústicos — picos de energia na banda calibrada 2,6–3,2 kHz (referência Áudio base/CEAES 2.m4a, pico ~2,89 kHz). Mesmo DetectionConfig em 75 arquivos, 104.742 h, 149962 eventos, 0 erros de processamento. Pipeline gerado em 2026-09-01T13:20:58.828375+00:00.</t>
+          <t>Este livro é PROVISÓRIO: serve para a aluna abrir, enviar por e-mail e usar no rascunho da tese. Não substitui a lista completa de eventos (output/resultado.xlsx, ~7 MB, gitignored). A aba Espectrogramas traz o recorte de escuta da madrugada com os picos marcados (validação humana). Não há um PNG por evento do lote (isso seriam ~150 mil imagens).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="78" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>O que NÃO afirmar</t>
+          <t>O que os números são</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Não são 149 962 machos, indivíduos ou pererecas. Um macho gera muitos eventos; dois machos no mesmo pitch podem virar um. Qualquer energia na banda acima do limiar vira evento (inseto, gravador, outra espécie). Não se comprovou espécie até de manhã. max_simultaneous = 2 é teto estrutural da banda de 600 Hz com separação de 400 Hz, não um censo. A Fase 3 (Claude) não foi usada.</t>
+          <t>Contagem automática de eventos acústicos — picos de energia na banda calibrada 2,6–3,2 kHz (referência Áudio base/CEAES 2.m4a, pico ~2,89 kHz). Mesmo DetectionConfig em 75 arquivos, 104.742 h, 149962 eventos, 0 erros de processamento. Pipeline gerado em 2026-09-01T13:20:58.828375+00:00.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="78" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Gráficos hora / mês</t>
+          <t>O que NÃO afirmar</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>A hora/mês é a do INÍCIO do arquivo (nome RYYYYMMDD-HHMMSS), não o relógio de cada canto. Sete MP3s (campanhas 12_09_25 e 15_08_25) não têm data no nome: 50 170 eventos entram no total e saem dos gráficos. Zeros às 11–13 h = nenhum WAV a começar nessa hora, não «zero canto». Agosto/setembro vazios nos gráficos pelas mesmas MP3s.</t>
+          <t>Não são 149 962 machos, indivíduos ou pererecas. Um macho gera muitos eventos; dois machos no mesmo pitch podem virar um. Qualquer energia na banda acima do limiar vira evento (inseto, gravador, outra espécie). Não se comprovou espécie até de manhã. max_simultaneous = 2 é teto estrutural da banda de 600 Hz com separação de 400 Hz, não um censo. A Fase 3 (Claude) não foi usada.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="78" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Próximo passo</t>
+          <t>Gráficos hora / mês</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Escuta humana do recorte já escolhido (aba Ouvir): pasta «10_10_25 açude 1», ficheiro R20241012-041002.WAV, gravado em 2024-10-12T04:10:02. Seek 30:45 (1845 s), ouvir 60 s até 31:45. Relógio de campo 04:40:47–04:41:47. O detector marcou 64 eventos curtos (~0.1 s), mediana ~2918 Hz (CEAES 2 ~2.89 kHz). Comparar com Áudio base/CEAES 2.m4a. NÃO começar pelo ficheiro da manhã R20241012-091022.WAV (09:10, o mais denso); só depois de o recorte da madrugada soar a rã.</t>
+          <t>A hora/mês é a do INÍCIO do arquivo (nome RYYYYMMDD-HHMMSS), não o relógio de cada canto. Sete MP3s (campanhas 12_09_25 e 15_08_25) não têm data no nome: 50 170 eventos entram no total e saem dos gráficos. Zeros às 11–13 h = nenhum WAV a começar nessa hora, não «zero canto». Agosto/setembro vazios nos gráficos pelas mesmas MP3s.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="78" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Documentos</t>
+          <t>Próximo passo</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>O que a tese pode afirmar: docs/PRECISAO_E_LIMITES.md. Como ler Excel/JSON completos: docs/COMO_LER_OS_RESULTADOS.md. Parâmetros: aba Parâmetros e src/bioacoustics/config.py. Totais enxutos: reports/campo_resumo.json. PNG de validação: aba Espectrogramas e reports/espectrogramas/.</t>
+          <t>Escuta humana do recorte já escolhido (aba Ouvir): pasta «10_10_25 açude 1», ficheiro R20241012-041002.WAV, gravado em 2024-10-12T04:10:02. Seek 30:45 (1845 s), ouvir 60 s até 31:45. Relógio de campo 04:40:47–04:41:47. O detector marcou 64 eventos curtos (~0.1 s), mediana ~2918 Hz (CEAES 2 ~2.89 kHz). Comparar com Áudio base/CEAES 2.m4a. NÃO começar pelo ficheiro da manhã R20241012-091022.WAV (09:10, o mais denso); só depois de o recorte da madrugada soar a rã.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="78" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
+          <t>Documentos</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>O que a tese pode afirmar: docs/PRECISAO_E_LIMITES.md. Como ler Excel/JSON completos: docs/COMO_LER_OS_RESULTADOS.md. Parâmetros: aba Parâmetros e src/bioacoustics/config.py. Totais enxutos: reports/campo_resumo.json. PNG de validação: aba Espectrogramas e reports/espectrogramas/.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="78" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
           <t>Como regenerar</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>python3 scripts/export_relatorio_provisorio.py  (gerado 2026-09-02 13:04 UTC). 64 eventos do recorte listados na aba Ouvir (extraídos de output/resultado.json).</t>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>python3 scripts/export_relatorio_provisorio.py  (gerado 2026-09-02 18:22 UTC). Lista dos 64 eventos do recorte ausente: rode o script na máquina com output/resultado.json para a preencher.</t>
         </is>
       </c>
     </row>
@@ -1393,7 +1433,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Pastas de açude 1. «15/08 açude 2 (esse nao precisa)» e «Áudio base» não entram. Campanhas só com MP3s não têm recorded_at.</t>
+          <t>Pastas de açude 1. «Eventos (soma)» = total de picos na campanha; «Eventos/h (média)» = média por arquivo (não é densidade horária do gráfico). MP3s sem data no nome ficam destacados.</t>
         </is>
       </c>
       <c r="B2" s="7" t="n"/>
@@ -1416,7 +1456,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Eventos</t>
+          <t>Eventos (soma)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1426,7 +1466,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Eventos/h</t>
+          <t>Eventos/h (média)</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -3845,7 +3885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4181,10 +4221,18 @@
       </c>
       <c r="C27" s="9" t="inlineStr"/>
     </row>
+    <row r="29">
+      <c r="A29" s="27" t="inlineStr">
+        <is>
+          <t>Pico: 05h — 7.181 eventos (início de arquivo neste bloco)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A29:F29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4198,7 +4246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4422,10 +4470,18 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>Pico: 10 out — 58.743 eventos (início de arquivo neste bloco)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4439,7 +4495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4634,1610 +4690,10 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B15" s="15" t="n">
-        <v>1845.339</v>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>04:40:47</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="n">
-        <v>3090</v>
-      </c>
-      <c r="E15" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F15" s="15" t="n">
-        <v>28.038</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B16" s="15" t="n">
-        <v>1845.85</v>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>04:40:47</t>
-        </is>
-      </c>
-      <c r="D16" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E16" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F16" s="15" t="n">
-        <v>74.901</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B17" s="15" t="n">
-        <v>1846.384</v>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>04:40:48</t>
-        </is>
-      </c>
-      <c r="D17" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E17" s="15" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="F17" s="15" t="n">
-        <v>42.902</v>
-      </c>
-      <c r="G17" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B18" s="15" t="n">
-        <v>1846.872</v>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>04:40:48</t>
-        </is>
-      </c>
-      <c r="D18" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E18" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F18" s="15" t="n">
-        <v>55.072</v>
-      </c>
-      <c r="G18" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B19" s="15" t="n">
-        <v>1847.452</v>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>04:40:49</t>
-        </is>
-      </c>
-      <c r="D19" s="11" t="n">
-        <v>3090</v>
-      </c>
-      <c r="E19" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F19" s="15" t="n">
-        <v>29.62</v>
-      </c>
-      <c r="G19" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B20" s="15" t="n">
-        <v>1848.009</v>
-      </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>04:40:50</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E20" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F20" s="15" t="n">
-        <v>56.337</v>
-      </c>
-      <c r="G20" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B21" s="15" t="n">
-        <v>1848.543</v>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>04:40:50</t>
-        </is>
-      </c>
-      <c r="D21" s="11" t="n">
-        <v>3143.8</v>
-      </c>
-      <c r="E21" s="15" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="F21" s="15" t="n">
-        <v>20.216</v>
-      </c>
-      <c r="G21" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B22" s="15" t="n">
-        <v>1849.078</v>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>04:40:51</t>
-        </is>
-      </c>
-      <c r="D22" s="11" t="n">
-        <v>2939.3</v>
-      </c>
-      <c r="E22" s="15" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="F22" s="15" t="n">
-        <v>33.363</v>
-      </c>
-      <c r="G22" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B23" s="15" t="n">
-        <v>1850.099</v>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>04:40:52</t>
-        </is>
-      </c>
-      <c r="D23" s="11" t="n">
-        <v>2939.3</v>
-      </c>
-      <c r="E23" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F23" s="15" t="n">
-        <v>41.71</v>
-      </c>
-      <c r="G23" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="B24" s="15" t="n">
-        <v>1850.61</v>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>04:40:52</t>
-        </is>
-      </c>
-      <c r="D24" s="11" t="n">
-        <v>3090</v>
-      </c>
-      <c r="E24" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F24" s="15" t="n">
-        <v>47.426</v>
-      </c>
-      <c r="G24" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="n">
-        <v>11</v>
-      </c>
-      <c r="B25" s="15" t="n">
-        <v>1851.121</v>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>04:40:53</t>
-        </is>
-      </c>
-      <c r="D25" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E25" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F25" s="15" t="n">
-        <v>60.029</v>
-      </c>
-      <c r="G25" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="B26" s="15" t="n">
-        <v>1851.678</v>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>04:40:53</t>
-        </is>
-      </c>
-      <c r="D26" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E26" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F26" s="15" t="n">
-        <v>36.121</v>
-      </c>
-      <c r="G26" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="n">
-        <v>13</v>
-      </c>
-      <c r="B27" s="15" t="n">
-        <v>1852.259</v>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>04:40:54</t>
-        </is>
-      </c>
-      <c r="D27" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E27" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F27" s="15" t="n">
-        <v>62.92</v>
-      </c>
-      <c r="G27" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="9" t="n">
-        <v>14</v>
-      </c>
-      <c r="B28" s="15" t="n">
-        <v>1853.118</v>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>04:40:55</t>
-        </is>
-      </c>
-      <c r="D28" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E28" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F28" s="15" t="n">
-        <v>49.537</v>
-      </c>
-      <c r="G28" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="n">
-        <v>15</v>
-      </c>
-      <c r="B29" s="15" t="n">
-        <v>1853.652</v>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>04:40:55</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E29" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F29" s="15" t="n">
-        <v>90.636</v>
-      </c>
-      <c r="G29" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="9" t="n">
-        <v>16</v>
-      </c>
-      <c r="B30" s="15" t="n">
-        <v>1854.697</v>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>04:40:56</t>
-        </is>
-      </c>
-      <c r="D30" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E30" s="15" t="n">
-        <v>0.302</v>
-      </c>
-      <c r="F30" s="15" t="n">
-        <v>83.167</v>
-      </c>
-      <c r="G30" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="n">
-        <v>17</v>
-      </c>
-      <c r="B31" s="15" t="n">
-        <v>1855.44</v>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>04:40:57</t>
-        </is>
-      </c>
-      <c r="D31" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E31" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F31" s="15" t="n">
-        <v>89.595</v>
-      </c>
-      <c r="G31" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="9" t="n">
-        <v>18</v>
-      </c>
-      <c r="B32" s="15" t="n">
-        <v>1855.951</v>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>04:40:57</t>
-        </is>
-      </c>
-      <c r="D32" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E32" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F32" s="15" t="n">
-        <v>32.234</v>
-      </c>
-      <c r="G32" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="9" t="n">
-        <v>19</v>
-      </c>
-      <c r="B33" s="15" t="n">
-        <v>1856.67</v>
-      </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>04:40:58</t>
-        </is>
-      </c>
-      <c r="D33" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E33" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F33" s="15" t="n">
-        <v>69.297</v>
-      </c>
-      <c r="G33" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="B34" s="15" t="n">
-        <v>1857.762</v>
-      </c>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t>04:40:59</t>
-        </is>
-      </c>
-      <c r="D34" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E34" s="15" t="n">
-        <v>1.207</v>
-      </c>
-      <c r="F34" s="15" t="n">
-        <v>75.598</v>
-      </c>
-      <c r="G34" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="9" t="n">
-        <v>21</v>
-      </c>
-      <c r="B35" s="15" t="n">
-        <v>1860.084</v>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>04:41:02</t>
-        </is>
-      </c>
-      <c r="D35" s="11" t="n">
-        <v>2799.3</v>
-      </c>
-      <c r="E35" s="15" t="n">
-        <v>0.929</v>
-      </c>
-      <c r="F35" s="15" t="n">
-        <v>12.49</v>
-      </c>
-      <c r="G35" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="B36" s="15" t="n">
-        <v>1861.802</v>
-      </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>04:41:03</t>
-        </is>
-      </c>
-      <c r="D36" s="11" t="n">
-        <v>2605.5</v>
-      </c>
-      <c r="E36" s="15" t="n">
-        <v>0.255</v>
-      </c>
-      <c r="F36" s="15" t="n">
-        <v>7.557</v>
-      </c>
-      <c r="G36" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="9" t="n">
-        <v>23</v>
-      </c>
-      <c r="B37" s="15" t="n">
-        <v>1863.335</v>
-      </c>
-      <c r="C37" s="9" t="inlineStr">
-        <is>
-          <t>04:41:05</t>
-        </is>
-      </c>
-      <c r="D37" s="11" t="n">
-        <v>2637.8</v>
-      </c>
-      <c r="E37" s="15" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="F37" s="15" t="n">
-        <v>18.349</v>
-      </c>
-      <c r="G37" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="9" t="n">
-        <v>24</v>
-      </c>
-      <c r="B38" s="15" t="n">
-        <v>1864.054</v>
-      </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>04:41:06</t>
-        </is>
-      </c>
-      <c r="D38" s="11" t="n">
-        <v>2745.5</v>
-      </c>
-      <c r="E38" s="15" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="F38" s="15" t="n">
-        <v>13.575</v>
-      </c>
-      <c r="G38" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="9" t="n">
-        <v>25</v>
-      </c>
-      <c r="B39" s="15" t="n">
-        <v>1865.262</v>
-      </c>
-      <c r="C39" s="9" t="inlineStr">
-        <is>
-          <t>04:41:07</t>
-        </is>
-      </c>
-      <c r="D39" s="11" t="n">
-        <v>2788.5</v>
-      </c>
-      <c r="E39" s="15" t="n">
-        <v>0.163</v>
-      </c>
-      <c r="F39" s="15" t="n">
-        <v>14.993</v>
-      </c>
-      <c r="G39" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="B40" s="15" t="n">
-        <v>1866.214</v>
-      </c>
-      <c r="C40" s="9" t="inlineStr">
-        <is>
-          <t>04:41:08</t>
-        </is>
-      </c>
-      <c r="D40" s="11" t="n">
-        <v>2734.7</v>
-      </c>
-      <c r="E40" s="15" t="n">
-        <v>0.139</v>
-      </c>
-      <c r="F40" s="15" t="n">
-        <v>12.565</v>
-      </c>
-      <c r="G40" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="9" t="n">
-        <v>27</v>
-      </c>
-      <c r="B41" s="15" t="n">
-        <v>1870.115</v>
-      </c>
-      <c r="C41" s="9" t="inlineStr">
-        <is>
-          <t>04:41:12</t>
-        </is>
-      </c>
-      <c r="D41" s="11" t="n">
-        <v>2982.3</v>
-      </c>
-      <c r="E41" s="15" t="n">
-        <v>2.02</v>
-      </c>
-      <c r="F41" s="15" t="n">
-        <v>29.627</v>
-      </c>
-      <c r="G41" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="9" t="n">
-        <v>28</v>
-      </c>
-      <c r="B42" s="15" t="n">
-        <v>1870.788</v>
-      </c>
-      <c r="C42" s="9" t="inlineStr">
-        <is>
-          <t>04:41:12</t>
-        </is>
-      </c>
-      <c r="D42" s="11" t="n">
-        <v>2637.8</v>
-      </c>
-      <c r="E42" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F42" s="15" t="n">
-        <v>16.208</v>
-      </c>
-      <c r="G42" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="9" t="n">
-        <v>29</v>
-      </c>
-      <c r="B43" s="15" t="n">
-        <v>1871.276</v>
-      </c>
-      <c r="C43" s="9" t="inlineStr">
-        <is>
-          <t>04:41:13</t>
-        </is>
-      </c>
-      <c r="D43" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E43" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F43" s="15" t="n">
-        <v>29.953</v>
-      </c>
-      <c r="G43" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="B44" s="15" t="n">
-        <v>1872.274</v>
-      </c>
-      <c r="C44" s="9" t="inlineStr">
-        <is>
-          <t>04:41:14</t>
-        </is>
-      </c>
-      <c r="D44" s="11" t="n">
-        <v>2960.8</v>
-      </c>
-      <c r="E44" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F44" s="15" t="n">
-        <v>31.616</v>
-      </c>
-      <c r="G44" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="9" t="n">
-        <v>31</v>
-      </c>
-      <c r="B45" s="15" t="n">
-        <v>1872.785</v>
-      </c>
-      <c r="C45" s="9" t="inlineStr">
-        <is>
-          <t>04:41:14</t>
-        </is>
-      </c>
-      <c r="D45" s="11" t="n">
-        <v>3165.4</v>
-      </c>
-      <c r="E45" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F45" s="15" t="n">
-        <v>14.018</v>
-      </c>
-      <c r="G45" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="9" t="n">
-        <v>32</v>
-      </c>
-      <c r="B46" s="15" t="n">
-        <v>1873.296</v>
-      </c>
-      <c r="C46" s="9" t="inlineStr">
-        <is>
-          <t>04:41:15</t>
-        </is>
-      </c>
-      <c r="D46" s="11" t="n">
-        <v>2799.3</v>
-      </c>
-      <c r="E46" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F46" s="15" t="n">
-        <v>30.776</v>
-      </c>
-      <c r="G46" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="9" t="n">
-        <v>33</v>
-      </c>
-      <c r="B47" s="15" t="n">
-        <v>1874.294</v>
-      </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>04:41:16</t>
-        </is>
-      </c>
-      <c r="D47" s="11" t="n">
-        <v>2820.8</v>
-      </c>
-      <c r="E47" s="15" t="n">
-        <v>0.604</v>
-      </c>
-      <c r="F47" s="15" t="n">
-        <v>37.613</v>
-      </c>
-      <c r="G47" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="9" t="n">
-        <v>34</v>
-      </c>
-      <c r="B48" s="15" t="n">
-        <v>1875.293</v>
-      </c>
-      <c r="C48" s="9" t="inlineStr">
-        <is>
-          <t>04:41:17</t>
-        </is>
-      </c>
-      <c r="D48" s="11" t="n">
-        <v>2702.4</v>
-      </c>
-      <c r="E48" s="15" t="n">
-        <v>0.139</v>
-      </c>
-      <c r="F48" s="15" t="n">
-        <v>30.969</v>
-      </c>
-      <c r="G48" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="9" t="n">
-        <v>35</v>
-      </c>
-      <c r="B49" s="15" t="n">
-        <v>1875.827</v>
-      </c>
-      <c r="C49" s="9" t="inlineStr">
-        <is>
-          <t>04:41:17</t>
-        </is>
-      </c>
-      <c r="D49" s="11" t="n">
-        <v>3176.1</v>
-      </c>
-      <c r="E49" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F49" s="15" t="n">
-        <v>17.356</v>
-      </c>
-      <c r="G49" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="9" t="n">
-        <v>36</v>
-      </c>
-      <c r="B50" s="15" t="n">
-        <v>1876.616</v>
-      </c>
-      <c r="C50" s="9" t="inlineStr">
-        <is>
-          <t>04:41:18</t>
-        </is>
-      </c>
-      <c r="D50" s="11" t="n">
-        <v>2788.5</v>
-      </c>
-      <c r="E50" s="15" t="n">
-        <v>0.232</v>
-      </c>
-      <c r="F50" s="15" t="n">
-        <v>42.013</v>
-      </c>
-      <c r="G50" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="9" t="n">
-        <v>37</v>
-      </c>
-      <c r="B51" s="15" t="n">
-        <v>1877.359</v>
-      </c>
-      <c r="C51" s="9" t="inlineStr">
-        <is>
-          <t>04:41:19</t>
-        </is>
-      </c>
-      <c r="D51" s="11" t="n">
-        <v>3079.2</v>
-      </c>
-      <c r="E51" s="15" t="n">
-        <v>0.325</v>
-      </c>
-      <c r="F51" s="15" t="n">
-        <v>10.056</v>
-      </c>
-      <c r="G51" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="9" t="n">
-        <v>38</v>
-      </c>
-      <c r="B52" s="15" t="n">
-        <v>1877.824</v>
-      </c>
-      <c r="C52" s="9" t="inlineStr">
-        <is>
-          <t>04:41:19</t>
-        </is>
-      </c>
-      <c r="D52" s="11" t="n">
-        <v>2724</v>
-      </c>
-      <c r="E52" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F52" s="15" t="n">
-        <v>27.472</v>
-      </c>
-      <c r="G52" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="9" t="n">
-        <v>39</v>
-      </c>
-      <c r="B53" s="15" t="n">
-        <v>1878.846</v>
-      </c>
-      <c r="C53" s="9" t="inlineStr">
-        <is>
-          <t>04:41:20</t>
-        </is>
-      </c>
-      <c r="D53" s="11" t="n">
-        <v>2917.7</v>
-      </c>
-      <c r="E53" s="15" t="n">
-        <v>0.5570000000000001</v>
-      </c>
-      <c r="F53" s="15" t="n">
-        <v>28.289</v>
-      </c>
-      <c r="G53" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="9" t="n">
-        <v>40</v>
-      </c>
-      <c r="B54" s="15" t="n">
-        <v>1879.356</v>
-      </c>
-      <c r="C54" s="9" t="inlineStr">
-        <is>
-          <t>04:41:21</t>
-        </is>
-      </c>
-      <c r="D54" s="11" t="n">
-        <v>2971.6</v>
-      </c>
-      <c r="E54" s="15" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="F54" s="15" t="n">
-        <v>27.926</v>
-      </c>
-      <c r="G54" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="9" t="n">
-        <v>41</v>
-      </c>
-      <c r="B55" s="15" t="n">
-        <v>1881.051</v>
-      </c>
-      <c r="C55" s="9" t="inlineStr">
-        <is>
-          <t>04:41:23</t>
-        </is>
-      </c>
-      <c r="D55" s="11" t="n">
-        <v>2767</v>
-      </c>
-      <c r="E55" s="15" t="n">
-        <v>1.463</v>
-      </c>
-      <c r="F55" s="15" t="n">
-        <v>35.758</v>
-      </c>
-      <c r="G55" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="9" t="n">
-        <v>42</v>
-      </c>
-      <c r="B56" s="15" t="n">
-        <v>1882.375</v>
-      </c>
-      <c r="C56" s="9" t="inlineStr">
-        <is>
-          <t>04:41:24</t>
-        </is>
-      </c>
-      <c r="D56" s="11" t="n">
-        <v>2777.8</v>
-      </c>
-      <c r="E56" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F56" s="15" t="n">
-        <v>32.074</v>
-      </c>
-      <c r="G56" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="9" t="n">
-        <v>43</v>
-      </c>
-      <c r="B57" s="15" t="n">
-        <v>1882.95</v>
-      </c>
-      <c r="C57" s="9" t="inlineStr">
-        <is>
-          <t>04:41:24</t>
-        </is>
-      </c>
-      <c r="D57" s="11" t="n">
-        <v>2724</v>
-      </c>
-      <c r="E57" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F57" s="15" t="n">
-        <v>23.89</v>
-      </c>
-      <c r="G57" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="9" t="n">
-        <v>44</v>
-      </c>
-      <c r="B58" s="15" t="n">
-        <v>1883.461</v>
-      </c>
-      <c r="C58" s="9" t="inlineStr">
-        <is>
-          <t>04:41:25</t>
-        </is>
-      </c>
-      <c r="D58" s="11" t="n">
-        <v>2767</v>
-      </c>
-      <c r="E58" s="15" t="n">
-        <v>0.186</v>
-      </c>
-      <c r="F58" s="15" t="n">
-        <v>33.822</v>
-      </c>
-      <c r="G58" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="9" t="n">
-        <v>45</v>
-      </c>
-      <c r="B59" s="15" t="n">
-        <v>1884.576</v>
-      </c>
-      <c r="C59" s="9" t="inlineStr">
-        <is>
-          <t>04:41:26</t>
-        </is>
-      </c>
-      <c r="D59" s="11" t="n">
-        <v>3046.9</v>
-      </c>
-      <c r="E59" s="15" t="n">
-        <v>0.186</v>
-      </c>
-      <c r="F59" s="15" t="n">
-        <v>16.543</v>
-      </c>
-      <c r="G59" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="9" t="n">
-        <v>46</v>
-      </c>
-      <c r="B60" s="15" t="n">
-        <v>1885.83</v>
-      </c>
-      <c r="C60" s="9" t="inlineStr">
-        <is>
-          <t>04:41:27</t>
-        </is>
-      </c>
-      <c r="D60" s="11" t="n">
-        <v>2874.7</v>
-      </c>
-      <c r="E60" s="15" t="n">
-        <v>1.277</v>
-      </c>
-      <c r="F60" s="15" t="n">
-        <v>24.839</v>
-      </c>
-      <c r="G60" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="9" t="n">
-        <v>47</v>
-      </c>
-      <c r="B61" s="15" t="n">
-        <v>1887.014</v>
-      </c>
-      <c r="C61" s="9" t="inlineStr">
-        <is>
-          <t>04:41:29</t>
-        </is>
-      </c>
-      <c r="D61" s="11" t="n">
-        <v>2928.5</v>
-      </c>
-      <c r="E61" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F61" s="15" t="n">
-        <v>24.112</v>
-      </c>
-      <c r="G61" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="9" t="n">
-        <v>48</v>
-      </c>
-      <c r="B62" s="15" t="n">
-        <v>1888.152</v>
-      </c>
-      <c r="C62" s="9" t="inlineStr">
-        <is>
-          <t>04:41:30</t>
-        </is>
-      </c>
-      <c r="D62" s="11" t="n">
-        <v>2745.5</v>
-      </c>
-      <c r="E62" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F62" s="15" t="n">
-        <v>17.237</v>
-      </c>
-      <c r="G62" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="9" t="n">
-        <v>49</v>
-      </c>
-      <c r="B63" s="15" t="n">
-        <v>1888.732</v>
-      </c>
-      <c r="C63" s="9" t="inlineStr">
-        <is>
-          <t>04:41:30</t>
-        </is>
-      </c>
-      <c r="D63" s="11" t="n">
-        <v>2713.2</v>
-      </c>
-      <c r="E63" s="15" t="n">
-        <v>0.998</v>
-      </c>
-      <c r="F63" s="15" t="n">
-        <v>21.434</v>
-      </c>
-      <c r="G63" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="9" t="n">
-        <v>50</v>
-      </c>
-      <c r="B64" s="15" t="n">
-        <v>1890.66</v>
-      </c>
-      <c r="C64" s="9" t="inlineStr">
-        <is>
-          <t>04:41:32</t>
-        </is>
-      </c>
-      <c r="D64" s="11" t="n">
-        <v>2799.3</v>
-      </c>
-      <c r="E64" s="15" t="n">
-        <v>0.604</v>
-      </c>
-      <c r="F64" s="15" t="n">
-        <v>29.823</v>
-      </c>
-      <c r="G64" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="9" t="n">
-        <v>51</v>
-      </c>
-      <c r="B65" s="15" t="n">
-        <v>1891.728</v>
-      </c>
-      <c r="C65" s="9" t="inlineStr">
-        <is>
-          <t>04:41:33</t>
-        </is>
-      </c>
-      <c r="D65" s="11" t="n">
-        <v>2767</v>
-      </c>
-      <c r="E65" s="15" t="n">
-        <v>0.604</v>
-      </c>
-      <c r="F65" s="15" t="n">
-        <v>22.563</v>
-      </c>
-      <c r="G65" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="9" t="n">
-        <v>52</v>
-      </c>
-      <c r="B66" s="15" t="n">
-        <v>1892.796</v>
-      </c>
-      <c r="C66" s="9" t="inlineStr">
-        <is>
-          <t>04:41:34</t>
-        </is>
-      </c>
-      <c r="D66" s="11" t="n">
-        <v>2777.8</v>
-      </c>
-      <c r="E66" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F66" s="15" t="n">
-        <v>37.032</v>
-      </c>
-      <c r="G66" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="9" t="n">
-        <v>53</v>
-      </c>
-      <c r="B67" s="15" t="n">
-        <v>1893.817</v>
-      </c>
-      <c r="C67" s="9" t="inlineStr">
-        <is>
-          <t>04:41:35</t>
-        </is>
-      </c>
-      <c r="D67" s="11" t="n">
-        <v>2756.2</v>
-      </c>
-      <c r="E67" s="15" t="n">
-        <v>0.604</v>
-      </c>
-      <c r="F67" s="15" t="n">
-        <v>39.972</v>
-      </c>
-      <c r="G67" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="9" t="n">
-        <v>54</v>
-      </c>
-      <c r="B68" s="15" t="n">
-        <v>1894.886</v>
-      </c>
-      <c r="C68" s="9" t="inlineStr">
-        <is>
-          <t>04:41:36</t>
-        </is>
-      </c>
-      <c r="D68" s="11" t="n">
-        <v>2767</v>
-      </c>
-      <c r="E68" s="15" t="n">
-        <v>0.163</v>
-      </c>
-      <c r="F68" s="15" t="n">
-        <v>31.216</v>
-      </c>
-      <c r="G68" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="9" t="n">
-        <v>55</v>
-      </c>
-      <c r="B69" s="15" t="n">
-        <v>1895.443</v>
-      </c>
-      <c r="C69" s="9" t="inlineStr">
-        <is>
-          <t>04:41:37</t>
-        </is>
-      </c>
-      <c r="D69" s="11" t="n">
-        <v>3068.5</v>
-      </c>
-      <c r="E69" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F69" s="15" t="n">
-        <v>39.844</v>
-      </c>
-      <c r="G69" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="9" t="n">
-        <v>56</v>
-      </c>
-      <c r="B70" s="15" t="n">
-        <v>1895.977</v>
-      </c>
-      <c r="C70" s="9" t="inlineStr">
-        <is>
-          <t>04:41:37</t>
-        </is>
-      </c>
-      <c r="D70" s="11" t="n">
-        <v>2713.2</v>
-      </c>
-      <c r="E70" s="15" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="F70" s="15" t="n">
-        <v>29.673</v>
-      </c>
-      <c r="G70" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="9" t="n">
-        <v>57</v>
-      </c>
-      <c r="B71" s="15" t="n">
-        <v>1896.488</v>
-      </c>
-      <c r="C71" s="9" t="inlineStr">
-        <is>
-          <t>04:41:38</t>
-        </is>
-      </c>
-      <c r="D71" s="11" t="n">
-        <v>2767</v>
-      </c>
-      <c r="E71" s="15" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="F71" s="15" t="n">
-        <v>22.536</v>
-      </c>
-      <c r="G71" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="9" t="n">
-        <v>58</v>
-      </c>
-      <c r="B72" s="15" t="n">
-        <v>1898.02</v>
-      </c>
-      <c r="C72" s="9" t="inlineStr">
-        <is>
-          <t>04:41:40</t>
-        </is>
-      </c>
-      <c r="D72" s="11" t="n">
-        <v>2831.6</v>
-      </c>
-      <c r="E72" s="15" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="F72" s="15" t="n">
-        <v>18.32</v>
-      </c>
-      <c r="G72" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="9" t="n">
-        <v>59</v>
-      </c>
-      <c r="B73" s="15" t="n">
-        <v>1898.903</v>
-      </c>
-      <c r="C73" s="9" t="inlineStr">
-        <is>
-          <t>04:41:40</t>
-        </is>
-      </c>
-      <c r="D73" s="11" t="n">
-        <v>2745.5</v>
-      </c>
-      <c r="E73" s="15" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="F73" s="15" t="n">
-        <v>13.27</v>
-      </c>
-      <c r="G73" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="9" t="n">
-        <v>60</v>
-      </c>
-      <c r="B74" s="15" t="n">
-        <v>1899.53</v>
-      </c>
-      <c r="C74" s="9" t="inlineStr">
-        <is>
-          <t>04:41:41</t>
-        </is>
-      </c>
-      <c r="D74" s="11" t="n">
-        <v>2745.5</v>
-      </c>
-      <c r="E74" s="15" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F74" s="15" t="n">
-        <v>12.409</v>
-      </c>
-      <c r="G74" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="9" t="n">
-        <v>61</v>
-      </c>
-      <c r="B75" s="15" t="n">
-        <v>1900.528</v>
-      </c>
-      <c r="C75" s="9" t="inlineStr">
-        <is>
-          <t>04:41:42</t>
-        </is>
-      </c>
-      <c r="D75" s="11" t="n">
-        <v>2745.5</v>
-      </c>
-      <c r="E75" s="15" t="n">
-        <v>0.209</v>
-      </c>
-      <c r="F75" s="15" t="n">
-        <v>41.317</v>
-      </c>
-      <c r="G75" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="9" t="n">
-        <v>62</v>
-      </c>
-      <c r="B76" s="15" t="n">
-        <v>1902.618</v>
-      </c>
-      <c r="C76" s="9" t="inlineStr">
-        <is>
-          <t>04:41:44</t>
-        </is>
-      </c>
-      <c r="D76" s="11" t="n">
-        <v>2767</v>
-      </c>
-      <c r="E76" s="15" t="n">
-        <v>1.138</v>
-      </c>
-      <c r="F76" s="15" t="n">
-        <v>39.177</v>
-      </c>
-      <c r="G76" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="9" t="n">
-        <v>63</v>
-      </c>
-      <c r="B77" s="15" t="n">
-        <v>1903.129</v>
-      </c>
-      <c r="C77" s="9" t="inlineStr">
-        <is>
-          <t>04:41:45</t>
-        </is>
-      </c>
-      <c r="D77" s="11" t="n">
-        <v>3090</v>
-      </c>
-      <c r="E77" s="15" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="F77" s="15" t="n">
-        <v>18.748</v>
-      </c>
-      <c r="G77" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="9" t="n">
-        <v>64</v>
-      </c>
-      <c r="B78" s="15" t="n">
-        <v>1904.684</v>
-      </c>
-      <c r="C78" s="9" t="inlineStr">
-        <is>
-          <t>04:41:46</t>
-        </is>
-      </c>
-      <c r="D78" s="11" t="n">
-        <v>2767</v>
-      </c>
-      <c r="E78" s="15" t="n">
-        <v>1.393</v>
-      </c>
-      <c r="F78" s="15" t="n">
-        <v>35.251</v>
-      </c>
-      <c r="G78" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="27" t="inlineStr">
-        <is>
-          <t>64 eventos no recorte 30:45–31:45 (ficheiro R20241012-041002.WAV). Duração mediana 0.116 s; frequência mediana 2917.7 Hz.</t>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>Lista dos 64 eventos indisponível neste ficheiro: output/resultado.json não estava presente (CI / máquina sem o JSON completo). Na cópia da tese gerada com o JSON local, esta tabela tem uma linha por evento (peak_time_s, relógio, frequência, duração, energia, n_callers). O recorte em si não muda.</t>
         </is>
       </c>
     </row>
@@ -6247,12 +4703,12 @@
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B5:G5"/>
-    <mergeCell ref="A79:G79"/>
     <mergeCell ref="B9:G9"/>
     <mergeCell ref="B8:G8"/>
     <mergeCell ref="B4:G4"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="B12:G12"/>
+    <mergeCell ref="A15:G15"/>
     <mergeCell ref="B7:G7"/>
     <mergeCell ref="B11:G11"/>
     <mergeCell ref="B6:G6"/>
@@ -6268,7 +4724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6297,55 +4753,42 @@
       <c r="C2" s="7" t="n"/>
       <c r="D2" s="7" t="n"/>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3" ht="36" customHeight="1">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>Como ler: fundo escuro = espectrograma; linha/círculo verde = pico do detector naquele instante (não re-detecção visual); eixo horizontal = tempo; vertical = kHz. Serve para ouvir+ver se o som parece o anúncio da espécie — não prova ID sozinho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Figura</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Ficheiro</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Legenda</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>reports/espectrogramas/R20241012-041002_30m45s.png</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>embutida</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>R20241012-041002.WAV — 30:45–31:45 (04:40) — picos de vocalização. Recorte de escuta já combinado (64 eventos, ~2,93 kHz). Círculos verdes = eventos do lote, não uma recontagem.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>reports/espectrogramas/R20241012-041002_pico_1854s.png</t>
+          <t>reports/espectrogramas/R20241012-041002_30m45s.png</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -6355,69 +4798,90 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Zoom ~8 s no pico mais forte deste minuto (~1853,65 s, 2928 Hz). Só para conferir a forma do canto; o método de contagem continua a ser a matriz numérica da STFT.</t>
+          <t>R20241012-041002.WAV — 30:45–31:45 (04:40) — picos de vocalização. Recorte de escuta já combinado (64 eventos, ~2,93 kHz). Círculos verdes = eventos do lote, não uma recontagem.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>reports/espectrogramas/R20241012-041002_pico_1854s.png</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>embutida</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Zoom ~8 s no pico mais forte deste minuto (~1853,65 s, 2928 Hz). Só para conferir a forma do canto; o método de contagem continua a ser a matriz numérica da STFT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>reports/espectrogramas/R20241012-091022_densest_60s.png</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>embutida</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>R20241012-091022.WAV — janela de 60 s mais densa — só depois da madrugada. Não começar a validação por este ficheiro.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="28" t="inlineStr">
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>Regenerar PNGs (máquina com o WAV de campo e output/resultado.json): python3 scripts/export_espectrogramas_validacao.py  depois  python3 scripts/export_relatorio_provisorio.py</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="29" t="inlineStr">
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
         <is>
           <t>R20241012-041002.WAV — 30:45–31:45 (04:40) — picos de vocalização. Recorte de escuta já combinado (64 eventos, ~2,93 kHz). Círculos verdes = eventos do lote, não uma recontagem.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="267" customHeight="1"/>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="29" t="inlineStr">
+    <row r="11" ht="267" customHeight="1"/>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="30" t="inlineStr">
         <is>
           <t>Zoom ~8 s no pico mais forte deste minuto (~1853,65 s, 2928 Hz). Só para conferir a forma do canto; o método de contagem continua a ser a matriz numérica da STFT.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="267" customHeight="1"/>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="29" t="inlineStr">
+    <row r="14" ht="267" customHeight="1"/>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>R20241012-091022.WAV — janela de 60 s mais densa — só depois da madrugada. Não começar a validação por este ficheiro.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="267" customHeight="1"/>
+    <row r="17" ht="267" customHeight="1"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A3:D3"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A13:D13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6475,7 +4939,7 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" s="31" t="inlineStr">
         <is>
           <t>sample_rate</t>
         </is>
@@ -6490,7 +4954,7 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="31" t="inlineStr">
         <is>
           <t>lowcut_hz</t>
         </is>
@@ -6505,7 +4969,7 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="A6" s="31" t="inlineStr">
         <is>
           <t>highcut_hz</t>
         </is>
@@ -6520,7 +4984,7 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="30" t="inlineStr">
+      <c r="A7" s="31" t="inlineStr">
         <is>
           <t>filter_order</t>
         </is>
@@ -6535,7 +4999,7 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="30" t="inlineStr">
+      <c r="A8" s="31" t="inlineStr">
         <is>
           <t>n_fft</t>
         </is>
@@ -6550,7 +5014,7 @@
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>hop_length</t>
         </is>
@@ -6565,7 +5029,7 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>use_noise_reduction</t>
         </is>
@@ -6582,7 +5046,7 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>noise_reduce_prop_decrease</t>
         </is>
@@ -6597,7 +5061,7 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>threshold_k</t>
         </is>
@@ -6612,7 +5076,7 @@
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="32" t="inlineStr">
         <is>
           <t>min_peak_distance_s</t>
         </is>
@@ -6620,14 +5084,14 @@
       <c r="B13" s="16" t="n">
         <v>0.15</v>
       </c>
-      <c r="C13" s="32" t="inlineStr">
+      <c r="C13" s="33" t="inlineStr">
         <is>
           <t>Declarado em DetectionConfig; NÃO é usado em detect_events.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>event_merge_gap_s</t>
         </is>
@@ -6642,7 +5106,7 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="30" t="inlineStr">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>min_event_duration_s</t>
         </is>
@@ -6657,7 +5121,7 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="30" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>freq_separation_hz</t>
         </is>
@@ -6672,7 +5136,7 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="30" t="inlineStr">
+      <c r="A17" s="31" t="inlineStr">
         <is>
           <t>caller_rel_height</t>
         </is>
@@ -6687,7 +5151,7 @@
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="30" t="inlineStr">
+      <c r="A18" s="31" t="inlineStr">
         <is>
           <t>edge_guard_s</t>
         </is>
@@ -6702,7 +5166,7 @@
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="30" t="inlineStr">
+      <c r="A19" s="31" t="inlineStr">
         <is>
           <t>chunk_duration_s</t>
         </is>
@@ -6717,7 +5181,7 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="30" t="inlineStr">
+      <c r="A20" s="31" t="inlineStr">
         <is>
           <t>chunk_overlap_s</t>
         </is>
@@ -6732,7 +5196,7 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="30" t="inlineStr">
+      <c r="A21" s="31" t="inlineStr">
         <is>
           <t>spectrogram_preview_s</t>
         </is>

</xml_diff>